<commit_message>
Check each source in a combined [S1, S2] citation (X9)
The real-source re-run showed that an answer citing "[S1, S2]" was recorded
with that whole bracket as one invalid label, so correct, supported answers
looked uncited. A bracket that lists only source labels now counts each one,
and the answer view links each valid source. Other bracket text is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/real-source-2026-10/real-source-test.xlsx
+++ b/docs/qa/real-source-2026-10/real-source-test.xlsx
@@ -30054,12 +30054,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Found during the spec 0007 re-run; not part of spec 0007.</t>
+          <t>Found during the spec 0007 re-run. validate_citations() now splits [S1, S2] into S1 and S2, and the answer view links each valid source. Covered by tests; recorded A1 answers keep the citations stored at the time.</t>
         </is>
       </c>
     </row>
@@ -30792,12 +30792,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Found during the spec 0007 re-run; not part of spec 0007.</t>
+          <t>Found during the spec 0007 re-run. validate_citations() now splits [S1, S2] into S1 and S2, and the answer view links each valid source. Covered by tests; recorded A1 answers keep the citations stored at the time.</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>

</xml_diff>